<commit_message>
Updated example files with area key
</commit_message>
<xml_diff>
--- a/PermitData/Halibut_ifq_EX.xlsx
+++ b/PermitData/Halibut_ifq_EX.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IFQ Reference" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4169,4 +4170,259 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Reference Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IFQ Area Reference:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2C - Southeast Alaska</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3A - Central Gulf of Alaska</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3B - Western Gulf of Alaska</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4A - Eastern Aleutian Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4B - Central/Western Aleutian Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4C - Pribilof Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4D - Northwestern Bering Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>4E - Bering Sea Flats</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Regulatory Areas for Halibut:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2C - Southeast Outside District</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3A - Eastern Gulf of Alaska</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3B - Central Gulf of Alaska</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>4A - Eastern Aleutians</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4B - Western Aleutians</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4C - Pribilof Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>4D - Northwestern Bering Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>4E - Bering Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Regulatory Areas for Sablefish:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AI - Aleutian Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BS - Bering Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CG - Central Gulf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SE - Southeast Outside</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>WG - Western Gulf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>WY - West Yakutat</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Vessel Categories:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>A - Vessels of any length</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>B - Vessels less than or equal to 60 feet in length</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>C - Vessels less than or equal to 35 feet in length</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>D - Vessels less than or equal to 60 feet in length, not a catcher/processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Block Status:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>B - Blocked quota share</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>U - Unblocked quota share</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>